<commit_message>
Add resource: Violet Directory
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -590,7 +590,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S162"/>
+  <dimension ref="A1:S163"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10154,9 +10154,68 @@
         <v>daytime resource center; homelessness; hot meals; showers; toiletries; laundry; lockers; mail service; phone charging; physical health care; mental health care; substance use care; employment training; job search; housing search; housing placement; veterans benefits; SNAP; Medical Assistance; financial support; legal support</v>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>Violet Directory</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Rainbow Health</v>
+      </c>
+      <c r="C163" t="str">
+        <v>LGBT+ Healthcare</v>
+      </c>
+      <c r="D163" t="str">
+        <v xml:space="preserve">Directories for LGBT+ friendly providers. Includes directories for providers specializing in HIV Care &amp; Prevention  and Aging. </v>
+      </c>
+      <c r="E163" t="str">
+        <v/>
+      </c>
+      <c r="F163" t="str">
+        <v/>
+      </c>
+      <c r="G163" t="str">
+        <v/>
+      </c>
+      <c r="H163" t="str">
+        <v/>
+      </c>
+      <c r="I163" t="str">
+        <v/>
+      </c>
+      <c r="J163" t="str">
+        <v/>
+      </c>
+      <c r="K163" t="str">
+        <v/>
+      </c>
+      <c r="L163" t="str">
+        <v>https://rainbowhealth.org/violet/</v>
+      </c>
+      <c r="M163" t="str">
+        <v/>
+      </c>
+      <c r="N163" t="str">
+        <v>Rainbow Health ceased operations in 2024. Directory is likely not maintained and subject to link rot.</v>
+      </c>
+      <c r="O163" t="str">
+        <v/>
+      </c>
+      <c r="P163" t="str">
+        <v>LGBT, Queer, Gay, HIV, AIDS, Aging, Directory, Rainbow, Violet</v>
+      </c>
+      <c r="Q163" t="str">
+        <v/>
+      </c>
+      <c r="R163" t="str">
+        <v>Health Care &amp; Clinics</v>
+      </c>
+      <c r="S163" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S162"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S163"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add resource: Hennepin ACT Team
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -590,7 +590,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S163"/>
+  <dimension ref="A1:S164"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10213,9 +10213,68 @@
         <v/>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>Hennepin ACT Team</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Mental Health Resources</v>
+      </c>
+      <c r="C164" t="str">
+        <v>ACT Team</v>
+      </c>
+      <c r="D164" t="str">
+        <v>Assertive Community Treatment</v>
+      </c>
+      <c r="E164" t="str">
+        <v/>
+      </c>
+      <c r="F164" t="str">
+        <v/>
+      </c>
+      <c r="G164" t="str">
+        <v>612-333-0331</v>
+      </c>
+      <c r="H164" t="str">
+        <v/>
+      </c>
+      <c r="I164" t="str">
+        <v>612-333-5614</v>
+      </c>
+      <c r="J164" t="str">
+        <v/>
+      </c>
+      <c r="K164" t="str">
+        <v/>
+      </c>
+      <c r="L164" t="str">
+        <v>https://www.mhresources.org/assertive-community-treatment-teams</v>
+      </c>
+      <c r="M164" t="str">
+        <v>2105 Minnehaha Ave, Minneapolis, MN 55404</v>
+      </c>
+      <c r="N164" t="str">
+        <v/>
+      </c>
+      <c r="O164" t="str">
+        <v/>
+      </c>
+      <c r="P164" t="str">
+        <v>Assertive, community, treatment, team</v>
+      </c>
+      <c r="Q164" t="str">
+        <v/>
+      </c>
+      <c r="R164" t="str">
+        <v>Mental Health &amp; Substance Use</v>
+      </c>
+      <c r="S164" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S163"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S164"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add resource: People Incorporated ACT Team
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -590,7 +590,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S164"/>
+  <dimension ref="A1:S165"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10272,9 +10272,68 @@
         <v/>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>People Incorporated ACT Team</v>
+      </c>
+      <c r="B165" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Mental Health Services</v>
+      </c>
+      <c r="D165" t="str">
+        <v/>
+      </c>
+      <c r="E165" t="str">
+        <v>Angela Mendez</v>
+      </c>
+      <c r="F165" t="str">
+        <v>angela.mendez@peopleincorporated.org</v>
+      </c>
+      <c r="G165" t="str">
+        <v>612-465-0105</v>
+      </c>
+      <c r="H165" t="str">
+        <v>651-774-0011</v>
+      </c>
+      <c r="I165" t="str">
+        <v>612-465-0107</v>
+      </c>
+      <c r="J165" t="str">
+        <v/>
+      </c>
+      <c r="K165" t="str">
+        <v/>
+      </c>
+      <c r="L165" t="str">
+        <v>https://peopleincorporated.org/programs/assertive-community-treatment-act/</v>
+      </c>
+      <c r="M165" t="str">
+        <v>: 2120 Park Ave. South, Minneapolis, MN 55404</v>
+      </c>
+      <c r="N165" t="str">
+        <v/>
+      </c>
+      <c r="O165" t="str">
+        <v/>
+      </c>
+      <c r="P165" t="str">
+        <v>ACT, People, Mental health</v>
+      </c>
+      <c r="Q165" t="str">
+        <v/>
+      </c>
+      <c r="R165" t="str">
+        <v>Health Care &amp; Clinics</v>
+      </c>
+      <c r="S165" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S164"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S165"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add resource: Intensive Residential Treatment Services
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -590,7 +590,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S165"/>
+  <dimension ref="A1:S166"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10331,9 +10331,68 @@
         <v/>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>Intensive Residential Treatment Services</v>
+      </c>
+      <c r="B166" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Mental Health Services</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Per website: Our Intensive Residential Treatment Services (IRTS) program integrates mental health, medical, and substance use care in a 24-hour, supervised setting. A step below hospitalization in our community-based system of care, these services help adults who need a high level of treatment and assistance in a structured environment. Individuals 18 years of age or older with a diagnosis of a mental illness who meet eligibility as designated by the Minnesota Department of Human Services (DHS).</v>
+      </c>
+      <c r="E166" t="str">
+        <v/>
+      </c>
+      <c r="F166" t="str">
+        <v>IRTS@peopleincorporated.org</v>
+      </c>
+      <c r="G166" t="str">
+        <v>651-774-0011</v>
+      </c>
+      <c r="H166" t="str">
+        <v/>
+      </c>
+      <c r="I166" t="str">
+        <v/>
+      </c>
+      <c r="J166" t="str">
+        <v/>
+      </c>
+      <c r="K166" t="str">
+        <v/>
+      </c>
+      <c r="L166" t="str">
+        <v>https://peopleincorporated.org/programs/intensive-residential-treatment-services-irts/</v>
+      </c>
+      <c r="M166" t="str">
+        <v/>
+      </c>
+      <c r="N166" t="str">
+        <v>Referral form : peopleincorporated.org/irts-referral-form/</v>
+      </c>
+      <c r="O166" t="str">
+        <v>Monday-Friday 7:00 AM–5:00 PM</v>
+      </c>
+      <c r="P166" t="str">
+        <v>residential, treatment, Mental health, in-patient</v>
+      </c>
+      <c r="Q166" t="str">
+        <v/>
+      </c>
+      <c r="R166" t="str">
+        <v>Mental Health &amp; Substance Use</v>
+      </c>
+      <c r="S166" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S165"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S166"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Edit resource: Intensive Residential Treatment Services -> People Incorporated Intensive Residential Treatment Services
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -10331,9 +10331,9 @@
         <v/>
       </c>
     </row>
-    <row r="166">
+    <row r="166" xml:space="preserve">
       <c r="A166" t="str">
-        <v>Intensive Residential Treatment Services</v>
+        <v>People Incorporated Intensive Residential Treatment Services</v>
       </c>
       <c r="B166" t="str">
         <v>People Incorporated</v>
@@ -10371,14 +10371,15 @@
       <c r="M166" t="str">
         <v/>
       </c>
-      <c r="N166" t="str">
-        <v>Referral form : peopleincorporated.org/irts-referral-form/</v>
+      <c r="N166" t="str" xml:space="preserve">
+        <v xml:space="preserve">Referral form: &lt;a href="https://peopleincorporated.org/irts-referral-form/"&gt;
+</v>
       </c>
       <c r="O166" t="str">
         <v>Monday-Friday 7:00 AM–5:00 PM</v>
       </c>
       <c r="P166" t="str">
-        <v>residential, treatment, Mental health, in-patient</v>
+        <v>residential, treatment, Mental health, in-patient, People, incorporated</v>
       </c>
       <c r="Q166" t="str">
         <v/>

</xml_diff>

<commit_message>
Edit resource: People Incorporated ACT Team
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -10272,7 +10272,7 @@
         <v/>
       </c>
     </row>
-    <row r="165">
+    <row r="165" xml:space="preserve">
       <c r="A165" t="str">
         <v>People Incorporated ACT Team</v>
       </c>
@@ -10283,7 +10283,7 @@
         <v>Mental Health Services</v>
       </c>
       <c r="D165" t="str">
-        <v/>
+        <v>An intensive, comprehensive outpatient treatment and rehabilitative mental health services program for adults (18+) with a primary diagnosis of schizophrenia, schizoaffective disorder, a major depressive disorder with psychotic features, bipolar disorder, or other psychotic disorders. The program provides support with services in co-occurring disorder treatment, family psychoeducation and support, housing access, medication education, and more.</v>
       </c>
       <c r="E165" t="str">
         <v>Angela Mendez</v>
@@ -10312,14 +10312,16 @@
       <c r="M165" t="str">
         <v>: 2120 Park Ave. South, Minneapolis, MN 55404</v>
       </c>
-      <c r="N165" t="str">
-        <v/>
+      <c r="N165" t="str" xml:space="preserve">
+        <v xml:space="preserve">Individuals need to be Hennepin County residents and engage with the ACT team 2-3 times per week. 
+Clients may be referred to programs and services by an insurance provider. Applicants with health coverage through a managed care organization must complete a chemical health assessment through their provider and obtain authorization prior to admission. A diagnostic assessment and discharge summaries from recent hospitalizations and/or previous psychiatric records are helpful to include with your referral.
+Referrals can come from anyone, even a self-referral, as long as a client is Hennepin County of Financial Responsibility (CFR).</v>
       </c>
       <c r="O165" t="str">
         <v/>
       </c>
       <c r="P165" t="str">
-        <v>ACT, People, Mental health</v>
+        <v>People, Mental health, Crisis, ACT, ASSERTIVE</v>
       </c>
       <c r="Q165" t="str">
         <v/>

</xml_diff>

<commit_message>
Edit resource: MN ACT
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -3738,13 +3738,13 @@
       <c r="F54" t="str">
         <v>dhs.dhhsd@state.mn.us</v>
       </c>
-      <c r="G54">
+      <c r="G54" t="str">
         <v>8006573663</v>
       </c>
       <c r="H54" t="str">
         <v>Videophone: 651-964-1514; Repair Office: 888-345-1725</v>
       </c>
-      <c r="I54">
+      <c r="I54" t="str">
         <v>6514317587</v>
       </c>
       <c r="J54" t="str">
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="P54" t="str">
-        <v>MN ACT, assistive technology, amplified phone, captioned phone, hearing loss, speech disability, phone accessibility</v>
+        <v>MN ACT, assistive technology, amplified phone, captioned phone, hearing loss, speech disability, phone accessibility, Phone, accessibility</v>
       </c>
       <c r="Q54" t="str">
         <v>MN ACT Program Guide|MN_ACT.pdf</v>
@@ -3775,7 +3775,7 @@
         <v>Seniors &amp; Disability</v>
       </c>
       <c r="S54" t="str">
-        <v>MN ACT; assistive technology; amplified phone; captioned phone; hearing loss; speech disability; phone accessibility</v>
+        <v/>
       </c>
     </row>
     <row r="55">

</xml_diff>

<commit_message>
Add resource: RADIAS Health Assertive Community Treatment
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -590,7 +590,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S166"/>
+  <dimension ref="A1:S167"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10393,9 +10393,68 @@
         <v/>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>RADIAS Health Assertive Community Treatment</v>
+      </c>
+      <c r="B167" t="str">
+        <v>RADIAS Health</v>
+      </c>
+      <c r="C167" t="str">
+        <v>ACT Team</v>
+      </c>
+      <c r="D167" t="str">
+        <v xml:space="preserve">Assertive Community Treatment (ACT) provides integrated mental health services treatment for individuals who have been diagnosed with thought disorders. Services include psychiatry, therapy, nursing, substance use disorder treatment, vocational services, case management, and peer recovery services. Teams partner with the individuals served and their natural supports to build the skills needed to manage their illness while also reaching their life goals. Common things teams help with include finding and maintaining housing, obtaining competitive employment, building social networks, and re-establishing relationships. Teams meet with people in their homes or community location of their choosing and provide services seven days a week, with crisis response services available 24 hours per day.  </v>
+      </c>
+      <c r="E167" t="str">
+        <v/>
+      </c>
+      <c r="F167" t="str">
+        <v>centralaccess@radiashealth.org</v>
+      </c>
+      <c r="G167" t="str">
+        <v>612-453-4010</v>
+      </c>
+      <c r="H167" t="str">
+        <v/>
+      </c>
+      <c r="I167" t="str">
+        <v>651-677-5714</v>
+      </c>
+      <c r="J167" t="str">
+        <v/>
+      </c>
+      <c r="K167" t="str">
+        <v/>
+      </c>
+      <c r="L167" t="str">
+        <v>https://www.radiashealth.org/programs/community-based-services/assertive-community-treatment/</v>
+      </c>
+      <c r="M167" t="str">
+        <v/>
+      </c>
+      <c r="N167" t="str">
+        <v>Referrals for all RADIAS programs are coordinated through their Central Access Team</v>
+      </c>
+      <c r="O167" t="str">
+        <v/>
+      </c>
+      <c r="P167" t="str">
+        <v>RADIAS, Health, ACT, Assertive Community Treatment, mental health</v>
+      </c>
+      <c r="Q167" t="str">
+        <v>ACT Referral FAQ|ACT-Referral-FAQ.pdf</v>
+      </c>
+      <c r="R167" t="str">
+        <v>Mental Health &amp; Substance Use</v>
+      </c>
+      <c r="S167" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S166"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S167"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Edit resource: RADIAS Health
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -10405,7 +10405,7 @@
         <v>Non-Profit Mental Health Services</v>
       </c>
       <c r="D167" t="str">
-        <v>Outpatient Individual and Group Therapy, Diagnostic Assessments, Medication Management, Dialectical Behavioral Therapy (DBT), Assertive Community Treatment (ACT), Forensic Assertive Community Treatment (FACT), Targeted Case Management, Waivered Services Case Management, Compass First Episode Psychosis Program, Community Competency Restoration, Intensive Residential Treatment Services (IRTS), Crisis Residential Services, Residential Support Services, Main Street Housing, Community Treatment Team Housing, Housing Support &amp; Navigation Programs, Homeless Outreach Services, Pharmacy Services, Professional Training Services</v>
+        <v>Mental Health non-profit offering various services including ACT,Youth ACT, out patient therapy, and emergency housing.</v>
       </c>
       <c r="E167" t="str">
         <v/>
@@ -11595,13 +11595,13 @@
         <v/>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>612-869-2411</v>
       </c>
       <c r="G8" t="str">
         <v/>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>https://www.radiashealth.org/programs/intensive-crisis-residential-treatment-services/reentry-house/</v>
       </c>
       <c r="I8" t="str">
         <v>5812 Lyndale Ave S, Minneapolis, MN 55419</v>

</xml_diff>

<commit_message>
Add resource: Veterans Services
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -589,7 +589,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S168"/>
+  <dimension ref="A1:S169"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10511,9 +10511,68 @@
         <v/>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>Veterans Services</v>
+      </c>
+      <c r="B169" t="str">
+        <v>Hennepin County</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Local CVSO Office</v>
+      </c>
+      <c r="D169" t="str">
+        <v/>
+      </c>
+      <c r="E169" t="str">
+        <v/>
+      </c>
+      <c r="F169" t="str">
+        <v>vetservices@hennepin.us</v>
+      </c>
+      <c r="G169" t="str">
+        <v xml:space="preserve"> 6123483300</v>
+      </c>
+      <c r="H169" t="str">
+        <v/>
+      </c>
+      <c r="I169" t="str">
+        <v>6123361373</v>
+      </c>
+      <c r="J169" t="str">
+        <v/>
+      </c>
+      <c r="K169" t="str">
+        <v/>
+      </c>
+      <c r="L169" t="str">
+        <v>https://www.hennepincounty.gov/services/assistance/veterans-services</v>
+      </c>
+      <c r="M169" t="str">
+        <v/>
+      </c>
+      <c r="N169" t="str">
+        <v/>
+      </c>
+      <c r="O169" t="str">
+        <v>Monday-Friday  8:00AM-4:30 PM</v>
+      </c>
+      <c r="P169" t="str">
+        <v>health, veteran, veterans, service, officer, VA, advocate, CVSO</v>
+      </c>
+      <c r="Q169" t="str">
+        <v>https://hcvetsvcs.powerappsportals.us/Intake-form/|link; Minnesota Association of Veteran Service Officers- Hennepin County|https://www.macvso.org/find-a-cvso.html?county=Hennepin+County|link</v>
+      </c>
+      <c r="R169" t="str">
+        <v>Benefits &amp; Insurance</v>
+      </c>
+      <c r="S169" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S168"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S169"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add resource: SpringPath Mental Health Services
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Screening Tools" sheetId="4" r:id="rId4"/>
     <sheet name="CAP-HC Contacts" sheetId="5" r:id="rId5"/>
     <sheet name="RADIAS Health Contacts" sheetId="6" r:id="rId6"/>
+    <sheet name="SpringPath Mental Heal Contacts" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Screening Tools'!A1:D22</definedName>
@@ -590,7 +591,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S169"/>
+  <dimension ref="A1:S170"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10571,9 +10572,68 @@
         <v/>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>SpringPath Mental Health Services</v>
+      </c>
+      <c r="B170" t="str">
+        <v>ResCare Minnesota, Inc.</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Mental Health Services</v>
+      </c>
+      <c r="D170" t="str">
+        <v>ACT, FACT, and IRTS service provider</v>
+      </c>
+      <c r="E170" t="str">
+        <v/>
+      </c>
+      <c r="F170" t="str">
+        <v/>
+      </c>
+      <c r="G170" t="str">
+        <v>7635376612</v>
+      </c>
+      <c r="H170" t="str">
+        <v/>
+      </c>
+      <c r="I170" t="str">
+        <v>7635377162</v>
+      </c>
+      <c r="J170" t="str">
+        <v/>
+      </c>
+      <c r="K170" t="str">
+        <v/>
+      </c>
+      <c r="L170" t="str">
+        <v>https://springpathmentalhealth.com/</v>
+      </c>
+      <c r="M170" t="str">
+        <v>6120 Earle Brown Drive, Suite 100 Brooklyn Center, MN 55430</v>
+      </c>
+      <c r="N170" t="str">
+        <v>Previously ResCare Minnesota</v>
+      </c>
+      <c r="O170" t="str">
+        <v/>
+      </c>
+      <c r="P170" t="str">
+        <v>ACT, Assertive, Community, Treatment, Mental, Health, ResCare, IRTS, Residential</v>
+      </c>
+      <c r="Q170" t="str">
+        <v/>
+      </c>
+      <c r="R170" t="str">
+        <v>Mental Health &amp; Substance Use</v>
+      </c>
+      <c r="S170" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S169"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S170"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11757,4 +11817,201 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SpringPath Mental Health Services — Sub-Contact Cards</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Each row is a related contact, viewable under the parent SpringPath Mental Health Services resource.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Parent Resource</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sub-Contact Name</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Services / Purpose</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Fax</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Email</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Website</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Location</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Hours / Availability</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Access Instructions</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SpringPath Mental Health Services</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Transitions on Broadway</v>
+      </c>
+      <c r="C5" t="str">
+        <v>IRTS</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>7635887626</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>3776 W Broadway, Minneapolis, MN 55422</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>SpringPath Mental Health Services</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Northwest Residence</v>
+      </c>
+      <c r="C6" t="str">
+        <v>IRTS</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>7635663650</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v>4408 69th Ave N, Brooklyn Center, MN 55429</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SpringPath Mental Health Services</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Phoenix Place</v>
+      </c>
+      <c r="C7" t="str">
+        <v>IRTS</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>7635368110</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v>4901 W BROADWAY AVE Crystal, MN 55429</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add resource: Simpson Housing Services
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -591,7 +591,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S170"/>
+  <dimension ref="A1:S171"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10631,9 +10631,68 @@
         <v/>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>Simpson Housing Services</v>
+      </c>
+      <c r="B171" t="str">
+        <v>Simpson Housing Services</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Housing &amp; Shelter</v>
+      </c>
+      <c r="D171" t="str">
+        <v/>
+      </c>
+      <c r="E171" t="str">
+        <v/>
+      </c>
+      <c r="F171" t="str">
+        <v/>
+      </c>
+      <c r="G171" t="str">
+        <v/>
+      </c>
+      <c r="H171" t="str">
+        <v/>
+      </c>
+      <c r="I171" t="str">
+        <v/>
+      </c>
+      <c r="J171" t="str">
+        <v/>
+      </c>
+      <c r="K171" t="str">
+        <v/>
+      </c>
+      <c r="L171" t="str">
+        <v>https://simpsonhousing.org</v>
+      </c>
+      <c r="M171" t="str">
+        <v>160 Glenwood Avenue Minneapolis, MN 55405</v>
+      </c>
+      <c r="N171" t="str">
+        <v/>
+      </c>
+      <c r="O171" t="str">
+        <v>Monday–Thursday 9AM–4PM</v>
+      </c>
+      <c r="P171" t="str">
+        <v/>
+      </c>
+      <c r="Q171" t="str">
+        <v/>
+      </c>
+      <c r="R171" t="str">
+        <v>Housing &amp; Shelter</v>
+      </c>
+      <c r="S171" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S170"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S171"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Edit resource: People Incorporated Intensive Residential Treatment Services
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -10335,7 +10335,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" xml:space="preserve">
+    <row r="166">
       <c r="A166" t="str">
         <v>People Incorporated Intensive Residential Treatment Services</v>
       </c>
@@ -10375,9 +10375,8 @@
       <c r="M166" t="str">
         <v/>
       </c>
-      <c r="N166" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;a href="https://peopleincorporated.org/irts-referral-form/" referral form&gt;_x000d_
-</v>
+      <c r="N166" t="str">
+        <v/>
       </c>
       <c r="O166" t="str">
         <v>Monday-Friday 7:00 AM–5:00 PM</v>
@@ -10386,7 +10385,7 @@
         <v>residential, treatment, Mental health, in-patient, People, incorporated</v>
       </c>
       <c r="Q166" t="str">
-        <v/>
+        <v>Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
       </c>
       <c r="R166" t="str">
         <v>Mental Health &amp; Substance Use</v>

</xml_diff>

<commit_message>
Add resource: People Incorporated
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -10,6 +10,7 @@
     <sheet name="CAP-HC Contacts" sheetId="5" r:id="rId5"/>
     <sheet name="RADIAS Health Contacts" sheetId="6" r:id="rId6"/>
     <sheet name="SpringPath Mental Heal Contacts" sheetId="7" r:id="rId7"/>
+    <sheet name="People Incorporated Contacts" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Screening Tools'!A1:D22</definedName>
@@ -591,7 +592,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S171"/>
+  <dimension ref="A1:S172"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10689,9 +10690,68 @@
         <v/>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="B172" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Non-Profit Mental Health Services</v>
+      </c>
+      <c r="D172" t="str">
+        <v>Non-Profit mental health provider with services including ACT, RCS, IRTS, outpatient programs, youth services, and case management.</v>
+      </c>
+      <c r="E172" t="str">
+        <v/>
+      </c>
+      <c r="F172" t="str">
+        <v>info@peopleincorporated.org</v>
+      </c>
+      <c r="G172" t="str">
+        <v>651-565-1564</v>
+      </c>
+      <c r="H172" t="str">
+        <v/>
+      </c>
+      <c r="I172" t="str">
+        <v/>
+      </c>
+      <c r="J172" t="str">
+        <v/>
+      </c>
+      <c r="K172" t="str">
+        <v/>
+      </c>
+      <c r="L172" t="str">
+        <v>https://peopleincorporated.org/</v>
+      </c>
+      <c r="M172" t="str">
+        <v>3000 Ames Crossing Road, Suite 600, Eagan, MN 55121</v>
+      </c>
+      <c r="N172" t="str">
+        <v/>
+      </c>
+      <c r="O172" t="str">
+        <v>Monday–Friday 7 am–5 pm</v>
+      </c>
+      <c r="P172" t="str">
+        <v>People, Incorporated, INC, ACT, IRTS, Assertive, Community, Treatment, Intensive, Residential, Housing, Case, Management</v>
+      </c>
+      <c r="Q172" t="str">
+        <v>IRTS Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
+      </c>
+      <c r="R172" t="str">
+        <v>Mental Health &amp; Substance Use</v>
+      </c>
+      <c r="S172" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S171"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S172"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -12072,4 +12132,157 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>People Incorporated — Sub-Contact Cards</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Each row is a related contact, viewable under the parent People Incorporated resource.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Parent Resource</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sub-Contact Name</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Services / Purpose</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Fax</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Email</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Website</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Location</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Hours / Availability</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Access Instructions</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Intensive Residential Treatment Services</v>
+      </c>
+      <c r="C5" t="str">
+        <v>IRTS</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>Per website: Our Intensive Residential Treatment Services (IRTS) program integrates mental health, medical, and substance use care in a 24-hour, supervised setting. A step below hospitalization in our community-based system of care, these services help adults who need a high level of treatment and assistance in a structured environment. Individuals 18 years of age or older with a diagnosis of a mental illness who meet eligibility as designated by the Minnesota Department of Human Services (DHS).</v>
+      </c>
+      <c r="F5" t="str">
+        <v>6517740011</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>IRTS@peopleincorporated.org</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://peopleincorporated.org/programs/intensive-residential-treatment-services-irts/</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Assertive Community Treatment</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ACT Team</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>An intensive, comprehensive outpatient treatment and rehabilitative mental health services program for adults (18+) with a primary diagnosis of schizophrenia, schizoaffective disorder, a major depressive disorder with psychotic features, bipolar disorder, or other psychotic disorders. The program provides support with services in co-occurring disorder treatment, family psychoeducation and support, housing access, medication education, and more.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>(612) 465-0105</v>
+      </c>
+      <c r="G6" t="str">
+        <v>(612) 465-0107</v>
+      </c>
+      <c r="H6" t="str">
+        <v>angela.mendez@peopleincorporated.org</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://peopleincorporated.org/programs/assertive-community-treatment-act/</v>
+      </c>
+      <c r="J6" t="str">
+        <v>2120 Park Ave. South Minneapolis, MN 55404</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v>Individuals need to be Hennepin County residents and engage with the ACT team 2-3 times per week. Clients may be referred to programs and services by an insurance provider. Applicants with health coverage through a managed care organization must complete a chemical health assessment through their provider and obtain authorization prior to admission. A diagnostic assessment and discharge summaries from recent hospitalizations and/or previous psychiatric records are helpful to include with your referral. Referrals can come from anyone, even a self-referral, as long as a client is Hennepin County of Financial Responsibility (CFR).</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Delete resource: People Incorporated ACT Team
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -592,7 +592,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S172"/>
+  <dimension ref="A1:S171"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10274,9 +10274,9 @@
         <v/>
       </c>
     </row>
-    <row r="165" xml:space="preserve">
+    <row r="165">
       <c r="A165" t="str">
-        <v>People Incorporated ACT Team</v>
+        <v>People Incorporated Intensive Residential Treatment Services</v>
       </c>
       <c r="B165" t="str">
         <v>People Incorporated</v>
@@ -10285,22 +10285,22 @@
         <v>Mental Health Services</v>
       </c>
       <c r="D165" t="str">
-        <v>An intensive, comprehensive outpatient treatment and rehabilitative mental health services program for adults (18+) with a primary diagnosis of schizophrenia, schizoaffective disorder, a major depressive disorder with psychotic features, bipolar disorder, or other psychotic disorders. The program provides support with services in co-occurring disorder treatment, family psychoeducation and support, housing access, medication education, and more.</v>
+        <v>Per website: Our Intensive Residential Treatment Services (IRTS) program integrates mental health, medical, and substance use care in a 24-hour, supervised setting. A step below hospitalization in our community-based system of care, these services help adults who need a high level of treatment and assistance in a structured environment. Individuals 18 years of age or older with a diagnosis of a mental illness who meet eligibility as designated by the Minnesota Department of Human Services (DHS).</v>
       </c>
       <c r="E165" t="str">
-        <v>Angela Mendez</v>
+        <v/>
       </c>
       <c r="F165" t="str">
-        <v>angela.mendez@peopleincorporated.org</v>
+        <v>IRTS@peopleincorporated.org</v>
       </c>
       <c r="G165" t="str">
-        <v>612-465-0105</v>
+        <v>651-774-0011</v>
       </c>
       <c r="H165" t="str">
-        <v>651-774-0011</v>
+        <v/>
       </c>
       <c r="I165" t="str">
-        <v>612-465-0107</v>
+        <v/>
       </c>
       <c r="J165" t="str">
         <v/>
@@ -10309,28 +10309,25 @@
         <v/>
       </c>
       <c r="L165" t="str">
-        <v>https://peopleincorporated.org/programs/assertive-community-treatment-act/</v>
+        <v>https://peopleincorporated.org/programs/intensive-residential-treatment-services-irts/</v>
       </c>
       <c r="M165" t="str">
-        <v>: 2120 Park Ave. South, Minneapolis, MN 55404</v>
-      </c>
-      <c r="N165" t="str" xml:space="preserve">
-        <v xml:space="preserve">Individuals need to be Hennepin County residents and engage with the ACT team 2-3 times per week. _x000d_
-_x000d_
-Clients may be referred to programs and services by an insurance provider. Applicants with health coverage through a managed care organization must complete a chemical health assessment through their provider and obtain authorization prior to admission. A diagnostic assessment and discharge summaries from recent hospitalizations and/or previous psychiatric records are helpful to include with your referral._x000d_
-Referrals can come from anyone, even a self-referral, as long as a client is Hennepin County of Financial Responsibility (CFR).</v>
+        <v/>
+      </c>
+      <c r="N165" t="str">
+        <v/>
       </c>
       <c r="O165" t="str">
-        <v/>
+        <v>Monday-Friday 7:00 AM–5:00 PM</v>
       </c>
       <c r="P165" t="str">
-        <v>People, Mental health, Crisis, ACT, ASSERTIVE</v>
+        <v>residential, treatment, Mental health, in-patient, People, incorporated</v>
       </c>
       <c r="Q165" t="str">
-        <v/>
+        <v>Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
       </c>
       <c r="R165" t="str">
-        <v>Health Care &amp; Clinics</v>
+        <v>Mental Health &amp; Substance Use</v>
       </c>
       <c r="S165" t="str">
         <v/>
@@ -10338,31 +10335,31 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>People Incorporated Intensive Residential Treatment Services</v>
+        <v>RADIAS Health</v>
       </c>
       <c r="B166" t="str">
-        <v>People Incorporated</v>
+        <v>RADIAS Health</v>
       </c>
       <c r="C166" t="str">
-        <v>Mental Health Services</v>
+        <v>Non-Profit Mental Health Services</v>
       </c>
       <c r="D166" t="str">
-        <v>Per website: Our Intensive Residential Treatment Services (IRTS) program integrates mental health, medical, and substance use care in a 24-hour, supervised setting. A step below hospitalization in our community-based system of care, these services help adults who need a high level of treatment and assistance in a structured environment. Individuals 18 years of age or older with a diagnosis of a mental illness who meet eligibility as designated by the Minnesota Department of Human Services (DHS).</v>
+        <v>Mental Health non-profit offering various services including ACT,Youth ACT, out patient therapy, and emergency housing.</v>
       </c>
       <c r="E166" t="str">
         <v/>
       </c>
       <c r="F166" t="str">
-        <v>IRTS@peopleincorporated.org</v>
+        <v>centralaccess@radiashealth.org</v>
       </c>
       <c r="G166" t="str">
-        <v>651-774-0011</v>
+        <v>612-453-4010</v>
       </c>
       <c r="H166" t="str">
         <v/>
       </c>
       <c r="I166" t="str">
-        <v/>
+        <v>651-677-5714</v>
       </c>
       <c r="J166" t="str">
         <v/>
@@ -10371,22 +10368,22 @@
         <v/>
       </c>
       <c r="L166" t="str">
-        <v>https://peopleincorporated.org/programs/intensive-residential-treatment-services-irts/</v>
+        <v>https://www.radiashealth.org/</v>
       </c>
       <c r="M166" t="str">
         <v/>
       </c>
       <c r="N166" t="str">
-        <v/>
+        <v>Referrals for all RADIAS programs are coordinated through their Central Access Team</v>
       </c>
       <c r="O166" t="str">
-        <v>Monday-Friday 7:00 AM–5:00 PM</v>
+        <v/>
       </c>
       <c r="P166" t="str">
-        <v>residential, treatment, Mental health, in-patient, People, incorporated</v>
+        <v>RADIAS, Health, ACT, Assertive Community Treatment, mental health, Youth, Pharmacy, Crisis, Residential</v>
       </c>
       <c r="Q166" t="str">
-        <v>Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
+        <v>RSS Referral Form|RSS-Referral.pdf; IRTS Referral Referral Form|RADIAS-IRTS-Referral.pdf; ACT Referral FAQ|ACT-Referral-FAQ-2.pdf; ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhAugPzsIjyMLyyiH7M7vAXvmHyHq2eqFFsU7eChprg6e07TbfawMdmc23vIqj4MGko*|link; Youth ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhBBuo-IVhRnsFoYhvNnm4hoxNvgY_OP57QRe6vHtGdQRGJkOLPW_JB1glr3-gbEuMc*|link</v>
       </c>
       <c r="R166" t="str">
         <v>Mental Health &amp; Substance Use</v>
@@ -10397,31 +10394,31 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>RADIAS Health</v>
+        <v>GoodRx</v>
       </c>
       <c r="B167" t="str">
-        <v>RADIAS Health</v>
+        <v>GoodRx</v>
       </c>
       <c r="C167" t="str">
-        <v>Non-Profit Mental Health Services</v>
+        <v>For-Profit Drug Discounter</v>
       </c>
       <c r="D167" t="str">
-        <v>Mental Health non-profit offering various services including ACT,Youth ACT, out patient therapy, and emergency housing.</v>
+        <v xml:space="preserve">GoodRx tracks prescription drug prices and provides users with drug savings coupons. </v>
       </c>
       <c r="E167" t="str">
         <v/>
       </c>
       <c r="F167" t="str">
-        <v>centralaccess@radiashealth.org</v>
+        <v/>
       </c>
       <c r="G167" t="str">
-        <v>612-453-4010</v>
+        <v/>
       </c>
       <c r="H167" t="str">
         <v/>
       </c>
       <c r="I167" t="str">
-        <v>651-677-5714</v>
+        <v/>
       </c>
       <c r="J167" t="str">
         <v/>
@@ -10430,25 +10427,25 @@
         <v/>
       </c>
       <c r="L167" t="str">
-        <v>https://www.radiashealth.org/</v>
+        <v>https://www.goodrx.com/</v>
       </c>
       <c r="M167" t="str">
         <v/>
       </c>
       <c r="N167" t="str">
-        <v>Referrals for all RADIAS programs are coordinated through their Central Access Team</v>
+        <v/>
       </c>
       <c r="O167" t="str">
         <v/>
       </c>
       <c r="P167" t="str">
-        <v>RADIAS, Health, ACT, Assertive Community Treatment, mental health, Youth, Pharmacy, Crisis, Residential</v>
+        <v>drugs, savings, prescription, coupons</v>
       </c>
       <c r="Q167" t="str">
-        <v>RSS Referral Form|RSS-Referral.pdf; IRTS Referral Referral Form|RADIAS-IRTS-Referral.pdf; ACT Referral FAQ|ACT-Referral-FAQ-2.pdf; ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhAugPzsIjyMLyyiH7M7vAXvmHyHq2eqFFsU7eChprg6e07TbfawMdmc23vIqj4MGko*|link; Youth ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhBBuo-IVhRnsFoYhvNnm4hoxNvgY_OP57QRe6vHtGdQRGJkOLPW_JB1glr3-gbEuMc*|link</v>
+        <v/>
       </c>
       <c r="R167" t="str">
-        <v>Mental Health &amp; Substance Use</v>
+        <v>Benefits &amp; Insurance</v>
       </c>
       <c r="S167" t="str">
         <v/>
@@ -10456,31 +10453,31 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>GoodRx</v>
+        <v>Veterans Services</v>
       </c>
       <c r="B168" t="str">
-        <v>GoodRx</v>
+        <v>Hennepin County</v>
       </c>
       <c r="C168" t="str">
-        <v>For-Profit Drug Discounter</v>
+        <v>Local CVSO Office</v>
       </c>
       <c r="D168" t="str">
-        <v xml:space="preserve">GoodRx tracks prescription drug prices and provides users with drug savings coupons. </v>
+        <v/>
       </c>
       <c r="E168" t="str">
         <v/>
       </c>
       <c r="F168" t="str">
-        <v/>
+        <v>vetservices@hennepin.us</v>
       </c>
       <c r="G168" t="str">
-        <v/>
+        <v xml:space="preserve"> 6123483300</v>
       </c>
       <c r="H168" t="str">
         <v/>
       </c>
       <c r="I168" t="str">
-        <v/>
+        <v>6123361373</v>
       </c>
       <c r="J168" t="str">
         <v/>
@@ -10489,7 +10486,7 @@
         <v/>
       </c>
       <c r="L168" t="str">
-        <v>https://www.goodrx.com/</v>
+        <v>https://www.hennepincounty.gov/services/assistance/veterans-services</v>
       </c>
       <c r="M168" t="str">
         <v/>
@@ -10498,13 +10495,13 @@
         <v/>
       </c>
       <c r="O168" t="str">
-        <v/>
+        <v>Monday-Friday  8:00AM-4:30 PM</v>
       </c>
       <c r="P168" t="str">
-        <v>drugs, savings, prescription, coupons</v>
+        <v>health, veteran, veterans, service, officer, VA, advocate, CVSO</v>
       </c>
       <c r="Q168" t="str">
-        <v/>
+        <v>https://hcvetsvcs.powerappsportals.us/Intake-form/|link; Minnesota Association of Veteran Service Officers- Hennepin County|https://www.macvso.org/find-a-cvso.html?county=Hennepin+County|link</v>
       </c>
       <c r="R168" t="str">
         <v>Benefits &amp; Insurance</v>
@@ -10515,31 +10512,31 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>Veterans Services</v>
+        <v>SpringPath Mental Health Services</v>
       </c>
       <c r="B169" t="str">
-        <v>Hennepin County</v>
+        <v>ResCare Minnesota, Inc.</v>
       </c>
       <c r="C169" t="str">
-        <v>Local CVSO Office</v>
+        <v>Mental Health Services</v>
       </c>
       <c r="D169" t="str">
-        <v/>
+        <v>ACT, FACT, and IRTS service provider</v>
       </c>
       <c r="E169" t="str">
         <v/>
       </c>
       <c r="F169" t="str">
-        <v>vetservices@hennepin.us</v>
+        <v/>
       </c>
       <c r="G169" t="str">
-        <v xml:space="preserve"> 6123483300</v>
+        <v>7635376612</v>
       </c>
       <c r="H169" t="str">
         <v/>
       </c>
       <c r="I169" t="str">
-        <v>6123361373</v>
+        <v>7635377162</v>
       </c>
       <c r="J169" t="str">
         <v/>
@@ -10548,25 +10545,25 @@
         <v/>
       </c>
       <c r="L169" t="str">
-        <v>https://www.hennepincounty.gov/services/assistance/veterans-services</v>
+        <v>https://springpathmentalhealth.com/</v>
       </c>
       <c r="M169" t="str">
-        <v/>
+        <v>6120 Earle Brown Drive, Suite 100 Brooklyn Center, MN 55430</v>
       </c>
       <c r="N169" t="str">
-        <v/>
+        <v>Previously ResCare Minnesota</v>
       </c>
       <c r="O169" t="str">
-        <v>Monday-Friday  8:00AM-4:30 PM</v>
+        <v/>
       </c>
       <c r="P169" t="str">
-        <v>health, veteran, veterans, service, officer, VA, advocate, CVSO</v>
+        <v>ACT, Assertive, Community, Treatment, Mental, Health, ResCare, IRTS, Residential</v>
       </c>
       <c r="Q169" t="str">
-        <v>https://hcvetsvcs.powerappsportals.us/Intake-form/|link; Minnesota Association of Veteran Service Officers- Hennepin County|https://www.macvso.org/find-a-cvso.html?county=Hennepin+County|link</v>
+        <v/>
       </c>
       <c r="R169" t="str">
-        <v>Benefits &amp; Insurance</v>
+        <v>Mental Health &amp; Substance Use</v>
       </c>
       <c r="S169" t="str">
         <v/>
@@ -10574,16 +10571,16 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>SpringPath Mental Health Services</v>
+        <v>Simpson Housing Services</v>
       </c>
       <c r="B170" t="str">
-        <v>ResCare Minnesota, Inc.</v>
+        <v>Simpson Housing Services</v>
       </c>
       <c r="C170" t="str">
-        <v>Mental Health Services</v>
+        <v>Housing &amp; Shelter</v>
       </c>
       <c r="D170" t="str">
-        <v>ACT, FACT, and IRTS service provider</v>
+        <v/>
       </c>
       <c r="E170" t="str">
         <v/>
@@ -10592,13 +10589,13 @@
         <v/>
       </c>
       <c r="G170" t="str">
-        <v>7635376612</v>
+        <v/>
       </c>
       <c r="H170" t="str">
         <v/>
       </c>
       <c r="I170" t="str">
-        <v>7635377162</v>
+        <v/>
       </c>
       <c r="J170" t="str">
         <v/>
@@ -10607,25 +10604,25 @@
         <v/>
       </c>
       <c r="L170" t="str">
-        <v>https://springpathmentalhealth.com/</v>
+        <v>https://simpsonhousing.org</v>
       </c>
       <c r="M170" t="str">
-        <v>6120 Earle Brown Drive, Suite 100 Brooklyn Center, MN 55430</v>
+        <v>160 Glenwood Avenue Minneapolis, MN 55405</v>
       </c>
       <c r="N170" t="str">
-        <v>Previously ResCare Minnesota</v>
+        <v/>
       </c>
       <c r="O170" t="str">
-        <v/>
+        <v>Monday–Thursday 9AM–4PM</v>
       </c>
       <c r="P170" t="str">
-        <v>ACT, Assertive, Community, Treatment, Mental, Health, ResCare, IRTS, Residential</v>
+        <v/>
       </c>
       <c r="Q170" t="str">
-        <v/>
+        <v>Simpson Brochure|Simpson-Brochure.pdf</v>
       </c>
       <c r="R170" t="str">
-        <v>Mental Health &amp; Substance Use</v>
+        <v>Housing &amp; Shelter</v>
       </c>
       <c r="S170" t="str">
         <v/>
@@ -10633,25 +10630,25 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>Simpson Housing Services</v>
+        <v>People Incorporated</v>
       </c>
       <c r="B171" t="str">
-        <v>Simpson Housing Services</v>
+        <v>People Incorporated</v>
       </c>
       <c r="C171" t="str">
-        <v>Housing &amp; Shelter</v>
+        <v>Non-Profit Mental Health Services</v>
       </c>
       <c r="D171" t="str">
-        <v/>
+        <v>Non-Profit mental health provider with services including ACT, RCS, IRTS, outpatient programs, youth services, and case management.</v>
       </c>
       <c r="E171" t="str">
         <v/>
       </c>
       <c r="F171" t="str">
-        <v/>
+        <v>info@peopleincorporated.org</v>
       </c>
       <c r="G171" t="str">
-        <v/>
+        <v>651-565-1564</v>
       </c>
       <c r="H171" t="str">
         <v/>
@@ -10666,92 +10663,33 @@
         <v/>
       </c>
       <c r="L171" t="str">
-        <v>https://simpsonhousing.org</v>
+        <v>https://peopleincorporated.org/</v>
       </c>
       <c r="M171" t="str">
-        <v>160 Glenwood Avenue Minneapolis, MN 55405</v>
+        <v>3000 Ames Crossing Road, Suite 600, Eagan, MN 55121</v>
       </c>
       <c r="N171" t="str">
         <v/>
       </c>
       <c r="O171" t="str">
-        <v>Monday–Thursday 9AM–4PM</v>
+        <v>Monday–Friday 7 am–5 pm</v>
       </c>
       <c r="P171" t="str">
-        <v/>
+        <v>People, Incorporated, INC, ACT, IRTS, Assertive, Community, Treatment, Intensive, Residential, Housing, Case, Management</v>
       </c>
       <c r="Q171" t="str">
-        <v>Simpson Brochure|Simpson-Brochure.pdf</v>
+        <v>IRTS Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
       </c>
       <c r="R171" t="str">
-        <v>Housing &amp; Shelter</v>
+        <v>Mental Health &amp; Substance Use</v>
       </c>
       <c r="S171" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="str">
-        <v>People Incorporated</v>
-      </c>
-      <c r="B172" t="str">
-        <v>People Incorporated</v>
-      </c>
-      <c r="C172" t="str">
-        <v>Non-Profit Mental Health Services</v>
-      </c>
-      <c r="D172" t="str">
-        <v>Non-Profit mental health provider with services including ACT, RCS, IRTS, outpatient programs, youth services, and case management.</v>
-      </c>
-      <c r="E172" t="str">
-        <v/>
-      </c>
-      <c r="F172" t="str">
-        <v>info@peopleincorporated.org</v>
-      </c>
-      <c r="G172" t="str">
-        <v>651-565-1564</v>
-      </c>
-      <c r="H172" t="str">
-        <v/>
-      </c>
-      <c r="I172" t="str">
-        <v/>
-      </c>
-      <c r="J172" t="str">
-        <v/>
-      </c>
-      <c r="K172" t="str">
-        <v/>
-      </c>
-      <c r="L172" t="str">
-        <v>https://peopleincorporated.org/</v>
-      </c>
-      <c r="M172" t="str">
-        <v>3000 Ames Crossing Road, Suite 600, Eagan, MN 55121</v>
-      </c>
-      <c r="N172" t="str">
-        <v/>
-      </c>
-      <c r="O172" t="str">
-        <v>Monday–Friday 7 am–5 pm</v>
-      </c>
-      <c r="P172" t="str">
-        <v>People, Incorporated, INC, ACT, IRTS, Assertive, Community, Treatment, Intensive, Residential, Housing, Case, Management</v>
-      </c>
-      <c r="Q172" t="str">
-        <v>IRTS Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
-      </c>
-      <c r="R172" t="str">
-        <v>Mental Health &amp; Substance Use</v>
-      </c>
-      <c r="S172" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S172"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S171"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Delete resource: People Incorporated Intensive Residential Treatment Services
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -592,7 +592,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S171"/>
+  <dimension ref="A1:S170"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10276,31 +10276,31 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>People Incorporated Intensive Residential Treatment Services</v>
+        <v>RADIAS Health</v>
       </c>
       <c r="B165" t="str">
-        <v>People Incorporated</v>
+        <v>RADIAS Health</v>
       </c>
       <c r="C165" t="str">
-        <v>Mental Health Services</v>
+        <v>Non-Profit Mental Health Services</v>
       </c>
       <c r="D165" t="str">
-        <v>Per website: Our Intensive Residential Treatment Services (IRTS) program integrates mental health, medical, and substance use care in a 24-hour, supervised setting. A step below hospitalization in our community-based system of care, these services help adults who need a high level of treatment and assistance in a structured environment. Individuals 18 years of age or older with a diagnosis of a mental illness who meet eligibility as designated by the Minnesota Department of Human Services (DHS).</v>
+        <v>Mental Health non-profit offering various services including ACT,Youth ACT, out patient therapy, and emergency housing.</v>
       </c>
       <c r="E165" t="str">
         <v/>
       </c>
       <c r="F165" t="str">
-        <v>IRTS@peopleincorporated.org</v>
+        <v>centralaccess@radiashealth.org</v>
       </c>
       <c r="G165" t="str">
-        <v>651-774-0011</v>
+        <v>612-453-4010</v>
       </c>
       <c r="H165" t="str">
         <v/>
       </c>
       <c r="I165" t="str">
-        <v/>
+        <v>651-677-5714</v>
       </c>
       <c r="J165" t="str">
         <v/>
@@ -10309,22 +10309,22 @@
         <v/>
       </c>
       <c r="L165" t="str">
-        <v>https://peopleincorporated.org/programs/intensive-residential-treatment-services-irts/</v>
+        <v>https://www.radiashealth.org/</v>
       </c>
       <c r="M165" t="str">
         <v/>
       </c>
       <c r="N165" t="str">
-        <v/>
+        <v>Referrals for all RADIAS programs are coordinated through their Central Access Team</v>
       </c>
       <c r="O165" t="str">
-        <v>Monday-Friday 7:00 AM–5:00 PM</v>
+        <v/>
       </c>
       <c r="P165" t="str">
-        <v>residential, treatment, Mental health, in-patient, People, incorporated</v>
+        <v>RADIAS, Health, ACT, Assertive Community Treatment, mental health, Youth, Pharmacy, Crisis, Residential</v>
       </c>
       <c r="Q165" t="str">
-        <v>Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
+        <v>RSS Referral Form|RSS-Referral.pdf; IRTS Referral Referral Form|RADIAS-IRTS-Referral.pdf; ACT Referral FAQ|ACT-Referral-FAQ-2.pdf; ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhAugPzsIjyMLyyiH7M7vAXvmHyHq2eqFFsU7eChprg6e07TbfawMdmc23vIqj4MGko*|link; Youth ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhBBuo-IVhRnsFoYhvNnm4hoxNvgY_OP57QRe6vHtGdQRGJkOLPW_JB1glr3-gbEuMc*|link</v>
       </c>
       <c r="R165" t="str">
         <v>Mental Health &amp; Substance Use</v>
@@ -10335,31 +10335,31 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>RADIAS Health</v>
+        <v>GoodRx</v>
       </c>
       <c r="B166" t="str">
-        <v>RADIAS Health</v>
+        <v>GoodRx</v>
       </c>
       <c r="C166" t="str">
-        <v>Non-Profit Mental Health Services</v>
+        <v>For-Profit Drug Discounter</v>
       </c>
       <c r="D166" t="str">
-        <v>Mental Health non-profit offering various services including ACT,Youth ACT, out patient therapy, and emergency housing.</v>
+        <v xml:space="preserve">GoodRx tracks prescription drug prices and provides users with drug savings coupons. </v>
       </c>
       <c r="E166" t="str">
         <v/>
       </c>
       <c r="F166" t="str">
-        <v>centralaccess@radiashealth.org</v>
+        <v/>
       </c>
       <c r="G166" t="str">
-        <v>612-453-4010</v>
+        <v/>
       </c>
       <c r="H166" t="str">
         <v/>
       </c>
       <c r="I166" t="str">
-        <v>651-677-5714</v>
+        <v/>
       </c>
       <c r="J166" t="str">
         <v/>
@@ -10368,25 +10368,25 @@
         <v/>
       </c>
       <c r="L166" t="str">
-        <v>https://www.radiashealth.org/</v>
+        <v>https://www.goodrx.com/</v>
       </c>
       <c r="M166" t="str">
         <v/>
       </c>
       <c r="N166" t="str">
-        <v>Referrals for all RADIAS programs are coordinated through their Central Access Team</v>
+        <v/>
       </c>
       <c r="O166" t="str">
         <v/>
       </c>
       <c r="P166" t="str">
-        <v>RADIAS, Health, ACT, Assertive Community Treatment, mental health, Youth, Pharmacy, Crisis, Residential</v>
+        <v>drugs, savings, prescription, coupons</v>
       </c>
       <c r="Q166" t="str">
-        <v>RSS Referral Form|RSS-Referral.pdf; IRTS Referral Referral Form|RADIAS-IRTS-Referral.pdf; ACT Referral FAQ|ACT-Referral-FAQ-2.pdf; ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhAugPzsIjyMLyyiH7M7vAXvmHyHq2eqFFsU7eChprg6e07TbfawMdmc23vIqj4MGko*|link; Youth ACT Referral Form|https://radiashealth.na4.adobesign.com/public/esignWidget?wid=CBFCIBAA3AAABLblqZhBBuo-IVhRnsFoYhvNnm4hoxNvgY_OP57QRe6vHtGdQRGJkOLPW_JB1glr3-gbEuMc*|link</v>
+        <v/>
       </c>
       <c r="R166" t="str">
-        <v>Mental Health &amp; Substance Use</v>
+        <v>Benefits &amp; Insurance</v>
       </c>
       <c r="S166" t="str">
         <v/>
@@ -10394,31 +10394,31 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>GoodRx</v>
+        <v>Veterans Services</v>
       </c>
       <c r="B167" t="str">
-        <v>GoodRx</v>
+        <v>Hennepin County</v>
       </c>
       <c r="C167" t="str">
-        <v>For-Profit Drug Discounter</v>
+        <v>Local CVSO Office</v>
       </c>
       <c r="D167" t="str">
-        <v xml:space="preserve">GoodRx tracks prescription drug prices and provides users with drug savings coupons. </v>
+        <v/>
       </c>
       <c r="E167" t="str">
         <v/>
       </c>
       <c r="F167" t="str">
-        <v/>
+        <v>vetservices@hennepin.us</v>
       </c>
       <c r="G167" t="str">
-        <v/>
+        <v xml:space="preserve"> 6123483300</v>
       </c>
       <c r="H167" t="str">
         <v/>
       </c>
       <c r="I167" t="str">
-        <v/>
+        <v>6123361373</v>
       </c>
       <c r="J167" t="str">
         <v/>
@@ -10427,7 +10427,7 @@
         <v/>
       </c>
       <c r="L167" t="str">
-        <v>https://www.goodrx.com/</v>
+        <v>https://www.hennepincounty.gov/services/assistance/veterans-services</v>
       </c>
       <c r="M167" t="str">
         <v/>
@@ -10436,13 +10436,13 @@
         <v/>
       </c>
       <c r="O167" t="str">
-        <v/>
+        <v>Monday-Friday  8:00AM-4:30 PM</v>
       </c>
       <c r="P167" t="str">
-        <v>drugs, savings, prescription, coupons</v>
+        <v>health, veteran, veterans, service, officer, VA, advocate, CVSO</v>
       </c>
       <c r="Q167" t="str">
-        <v/>
+        <v>https://hcvetsvcs.powerappsportals.us/Intake-form/|link; Minnesota Association of Veteran Service Officers- Hennepin County|https://www.macvso.org/find-a-cvso.html?county=Hennepin+County|link</v>
       </c>
       <c r="R167" t="str">
         <v>Benefits &amp; Insurance</v>
@@ -10453,31 +10453,31 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>Veterans Services</v>
+        <v>SpringPath Mental Health Services</v>
       </c>
       <c r="B168" t="str">
-        <v>Hennepin County</v>
+        <v>ResCare Minnesota, Inc.</v>
       </c>
       <c r="C168" t="str">
-        <v>Local CVSO Office</v>
+        <v>Mental Health Services</v>
       </c>
       <c r="D168" t="str">
-        <v/>
+        <v>ACT, FACT, and IRTS service provider</v>
       </c>
       <c r="E168" t="str">
         <v/>
       </c>
       <c r="F168" t="str">
-        <v>vetservices@hennepin.us</v>
+        <v/>
       </c>
       <c r="G168" t="str">
-        <v xml:space="preserve"> 6123483300</v>
+        <v>7635376612</v>
       </c>
       <c r="H168" t="str">
         <v/>
       </c>
       <c r="I168" t="str">
-        <v>6123361373</v>
+        <v>7635377162</v>
       </c>
       <c r="J168" t="str">
         <v/>
@@ -10486,25 +10486,25 @@
         <v/>
       </c>
       <c r="L168" t="str">
-        <v>https://www.hennepincounty.gov/services/assistance/veterans-services</v>
+        <v>https://springpathmentalhealth.com/</v>
       </c>
       <c r="M168" t="str">
-        <v/>
+        <v>6120 Earle Brown Drive, Suite 100 Brooklyn Center, MN 55430</v>
       </c>
       <c r="N168" t="str">
-        <v/>
+        <v>Previously ResCare Minnesota</v>
       </c>
       <c r="O168" t="str">
-        <v>Monday-Friday  8:00AM-4:30 PM</v>
+        <v/>
       </c>
       <c r="P168" t="str">
-        <v>health, veteran, veterans, service, officer, VA, advocate, CVSO</v>
+        <v>ACT, Assertive, Community, Treatment, Mental, Health, ResCare, IRTS, Residential</v>
       </c>
       <c r="Q168" t="str">
-        <v>https://hcvetsvcs.powerappsportals.us/Intake-form/|link; Minnesota Association of Veteran Service Officers- Hennepin County|https://www.macvso.org/find-a-cvso.html?county=Hennepin+County|link</v>
+        <v/>
       </c>
       <c r="R168" t="str">
-        <v>Benefits &amp; Insurance</v>
+        <v>Mental Health &amp; Substance Use</v>
       </c>
       <c r="S168" t="str">
         <v/>
@@ -10512,16 +10512,16 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>SpringPath Mental Health Services</v>
+        <v>Simpson Housing Services</v>
       </c>
       <c r="B169" t="str">
-        <v>ResCare Minnesota, Inc.</v>
+        <v>Simpson Housing Services</v>
       </c>
       <c r="C169" t="str">
-        <v>Mental Health Services</v>
+        <v>Housing &amp; Shelter</v>
       </c>
       <c r="D169" t="str">
-        <v>ACT, FACT, and IRTS service provider</v>
+        <v/>
       </c>
       <c r="E169" t="str">
         <v/>
@@ -10530,13 +10530,13 @@
         <v/>
       </c>
       <c r="G169" t="str">
-        <v>7635376612</v>
+        <v/>
       </c>
       <c r="H169" t="str">
         <v/>
       </c>
       <c r="I169" t="str">
-        <v>7635377162</v>
+        <v/>
       </c>
       <c r="J169" t="str">
         <v/>
@@ -10545,25 +10545,25 @@
         <v/>
       </c>
       <c r="L169" t="str">
-        <v>https://springpathmentalhealth.com/</v>
+        <v>https://simpsonhousing.org</v>
       </c>
       <c r="M169" t="str">
-        <v>6120 Earle Brown Drive, Suite 100 Brooklyn Center, MN 55430</v>
+        <v>160 Glenwood Avenue Minneapolis, MN 55405</v>
       </c>
       <c r="N169" t="str">
-        <v>Previously ResCare Minnesota</v>
+        <v/>
       </c>
       <c r="O169" t="str">
-        <v/>
+        <v>Monday–Thursday 9AM–4PM</v>
       </c>
       <c r="P169" t="str">
-        <v>ACT, Assertive, Community, Treatment, Mental, Health, ResCare, IRTS, Residential</v>
+        <v/>
       </c>
       <c r="Q169" t="str">
-        <v/>
+        <v>Simpson Brochure|Simpson-Brochure.pdf</v>
       </c>
       <c r="R169" t="str">
-        <v>Mental Health &amp; Substance Use</v>
+        <v>Housing &amp; Shelter</v>
       </c>
       <c r="S169" t="str">
         <v/>
@@ -10571,25 +10571,25 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>Simpson Housing Services</v>
+        <v>People Incorporated</v>
       </c>
       <c r="B170" t="str">
-        <v>Simpson Housing Services</v>
+        <v>People Incorporated</v>
       </c>
       <c r="C170" t="str">
-        <v>Housing &amp; Shelter</v>
+        <v>Non-Profit Mental Health Services</v>
       </c>
       <c r="D170" t="str">
-        <v/>
+        <v>Non-Profit mental health provider with services including ACT, RCS, IRTS, outpatient programs, youth services, and case management.</v>
       </c>
       <c r="E170" t="str">
         <v/>
       </c>
       <c r="F170" t="str">
-        <v/>
+        <v>info@peopleincorporated.org</v>
       </c>
       <c r="G170" t="str">
-        <v/>
+        <v>651-565-1564</v>
       </c>
       <c r="H170" t="str">
         <v/>
@@ -10604,92 +10604,33 @@
         <v/>
       </c>
       <c r="L170" t="str">
-        <v>https://simpsonhousing.org</v>
+        <v>https://peopleincorporated.org/</v>
       </c>
       <c r="M170" t="str">
-        <v>160 Glenwood Avenue Minneapolis, MN 55405</v>
+        <v>3000 Ames Crossing Road, Suite 600, Eagan, MN 55121</v>
       </c>
       <c r="N170" t="str">
         <v/>
       </c>
       <c r="O170" t="str">
-        <v>Monday–Thursday 9AM–4PM</v>
+        <v>Monday–Friday 7 am–5 pm</v>
       </c>
       <c r="P170" t="str">
-        <v/>
+        <v>People, Incorporated, INC, ACT, IRTS, Assertive, Community, Treatment, Intensive, Residential, Housing, Case, Management</v>
       </c>
       <c r="Q170" t="str">
-        <v>Simpson Brochure|Simpson-Brochure.pdf</v>
+        <v>IRTS Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
       </c>
       <c r="R170" t="str">
-        <v>Housing &amp; Shelter</v>
+        <v>Mental Health &amp; Substance Use</v>
       </c>
       <c r="S170" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="str">
-        <v>People Incorporated</v>
-      </c>
-      <c r="B171" t="str">
-        <v>People Incorporated</v>
-      </c>
-      <c r="C171" t="str">
-        <v>Non-Profit Mental Health Services</v>
-      </c>
-      <c r="D171" t="str">
-        <v>Non-Profit mental health provider with services including ACT, RCS, IRTS, outpatient programs, youth services, and case management.</v>
-      </c>
-      <c r="E171" t="str">
-        <v/>
-      </c>
-      <c r="F171" t="str">
-        <v>info@peopleincorporated.org</v>
-      </c>
-      <c r="G171" t="str">
-        <v>651-565-1564</v>
-      </c>
-      <c r="H171" t="str">
-        <v/>
-      </c>
-      <c r="I171" t="str">
-        <v/>
-      </c>
-      <c r="J171" t="str">
-        <v/>
-      </c>
-      <c r="K171" t="str">
-        <v/>
-      </c>
-      <c r="L171" t="str">
-        <v>https://peopleincorporated.org/</v>
-      </c>
-      <c r="M171" t="str">
-        <v>3000 Ames Crossing Road, Suite 600, Eagan, MN 55121</v>
-      </c>
-      <c r="N171" t="str">
-        <v/>
-      </c>
-      <c r="O171" t="str">
-        <v>Monday–Friday 7 am–5 pm</v>
-      </c>
-      <c r="P171" t="str">
-        <v>People, Incorporated, INC, ACT, IRTS, Assertive, Community, Treatment, Intensive, Residential, Housing, Case, Management</v>
-      </c>
-      <c r="Q171" t="str">
-        <v>IRTS Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
-      </c>
-      <c r="R171" t="str">
-        <v>Mental Health &amp; Substance Use</v>
-      </c>
-      <c r="S171" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S171"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S170"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Edit resource: People Incorporated
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -10580,7 +10580,7 @@
         <v>Non-Profit Mental Health Services</v>
       </c>
       <c r="D170" t="str">
-        <v>Non-Profit mental health provider with services including ACT, RCS, IRTS, outpatient programs, youth services, and case management.</v>
+        <v>Non-Profit mental health provider with services including ACT, RCS, IRTS, outpatient programs, youth services, Deaf and Hard of Hearing Services (DHHS), and case management.</v>
       </c>
       <c r="E170" t="str">
         <v/>
@@ -10601,7 +10601,7 @@
         <v/>
       </c>
       <c r="K170" t="str">
-        <v/>
+        <v>651-288-3463</v>
       </c>
       <c r="L170" t="str">
         <v>https://peopleincorporated.org/</v>
@@ -10619,7 +10619,7 @@
         <v>People, Incorporated, INC, ACT, IRTS, Assertive, Community, Treatment, Intensive, Residential, Housing, Case, Management</v>
       </c>
       <c r="Q170" t="str">
-        <v>IRTS Referral Form|https://peopleincorporated.org/irts-referral-form/|link</v>
+        <v>IRTS Referral Form|https://peopleincorporated.org/irts-referral-form/|link; Long Term Residential Services Referral Form|https://peopleincorporated.org/long-term-residential-services-referral-form/|link</v>
       </c>
       <c r="R170" t="str">
         <v>Mental Health &amp; Substance Use</v>
@@ -12015,7 +12015,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12159,9 +12159,97 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Residental Services</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Housing</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>https://peopleincorporated.org/programs/residential-services/</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>People Incorporated</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Access &amp; Recovery Center (ARC)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Outreach Team</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>Conntects people experiencing homelessness or housing instability with resources</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>ARCOutreachteam@peopleincorporated.org</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://peopleincorporated.org/programs/residential-services/access-recovery-center-arc-outreach-team/</v>
+      </c>
+      <c r="J8" t="str">
+        <v>317 York Avenue St. Paul, MN 55130</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add resource: St. Louis Park Housing Authority
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -592,7 +592,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S170"/>
+  <dimension ref="A1:S171"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10628,9 +10628,76 @@
         <v/>
       </c>
     </row>
+    <row r="171" xml:space="preserve">
+      <c r="A171" t="str">
+        <v>St. Louis Park Housing Authority</v>
+      </c>
+      <c r="B171" t="str">
+        <v>City of St. Louis Park</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Local government public housing</v>
+      </c>
+      <c r="D171" t="str" xml:space="preserve">
+        <v xml:space="preserve">The Public Housing Program provides clean, safe and affordable living environments for eligible low-income individuals and families. Those eligible for public housing pay 30% of their adjusted income for rent. 
+Public housing units are owned and managed by the St. Louis Park Housing Authority (HA). Current units within the city include:
+110 units in a low-rise apartment building (108 one-bedroom units and 2 two-bedroom units). This building is designated for general occupancy; however, a priority is given for elderly and disabled applicants.
+37 single-family homes (3 to 5 bedrooms) for families with children.
+12 two-bedroom apartment units located at Louisiana Court. These units are owned by Project for Pride in Living and managed by MetroPlains Management.</v>
+      </c>
+      <c r="E171" t="str">
+        <v/>
+      </c>
+      <c r="F171" t="str">
+        <v>waitinglist@stlouisparkmn.gov</v>
+      </c>
+      <c r="G171" t="str">
+        <v xml:space="preserve"> 9529242579</v>
+      </c>
+      <c r="H171" t="str">
+        <v/>
+      </c>
+      <c r="I171" t="str">
+        <v/>
+      </c>
+      <c r="J171" t="str">
+        <v/>
+      </c>
+      <c r="K171" t="str">
+        <v/>
+      </c>
+      <c r="L171" t="str">
+        <v>https://www.stlouisparkmn.gov/government/departments-divisions/housing/rental-assistance-housing-authority/public-housing</v>
+      </c>
+      <c r="M171" t="str">
+        <v>5005 Minnetonka Blvd, St Louis Park, MN 55416</v>
+      </c>
+      <c r="N171" t="str" xml:space="preserve">
+        <v xml:space="preserve">Applicants must meet eligibility requirements in order to qualify for public housing. Requirements include: 
+Meeting income guidelines at or below 80% area median income
+Meeting occupancy standards based on bedroom size
+Passing a rental screening process, including past rental history, criminal history check and review of credit history
+Applications for public housing are only accepted when the waiting list is open.</v>
+      </c>
+      <c r="O171" t="str">
+        <v/>
+      </c>
+      <c r="P171" t="str">
+        <v>Public, Housing, Rent, Income Adjusted</v>
+      </c>
+      <c r="Q171" t="str">
+        <v>Online Applicant Portal|https://housing-slpmn.securecafe.com/onlineleasing/st-louis-park-housing-authority/guestlogin.aspx?utm_nooverride=1&amp;propleadsource_1787017=portal&amp;_yTrackUser=NDQxOTk2MDc1MCMxOTIxNjg3ODkz-vrZNMJRdElM%253d&amp;_yTrackVisit=NzEzODI1NDIzNSMxNTc2NTU1NDc2-%252fhCtaYkSHf8%253d&amp;_yTrackReqDT=00371720261808|link; Housing Authority Website|https://housing.slpmn.us/|link; Housing Division Contact Directory|https://www.stlouisparkmn.gov/government/staff-directory/-selcat-19|link</v>
+      </c>
+      <c r="R171" t="str">
+        <v>Housing &amp; Shelter</v>
+      </c>
+      <c r="S171" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S170"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S171"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add resource: Day One
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -11,6 +11,7 @@
     <sheet name="RADIAS Health Contacts" sheetId="6" r:id="rId6"/>
     <sheet name="SpringPath Mental Heal Contacts" sheetId="7" r:id="rId7"/>
     <sheet name="People Incorporated Contacts" sheetId="8" r:id="rId8"/>
+    <sheet name="Day One Contacts" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Screening Tools'!A1:D22</definedName>
@@ -592,7 +593,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S171"/>
+  <dimension ref="A1:S172"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10695,9 +10696,68 @@
         <v/>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>Day One</v>
+      </c>
+      <c r="B172" t="str">
+        <v>Cornerstone MN</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Domestica Violence/Crime Victim Advocacy</v>
+      </c>
+      <c r="D172" t="str">
+        <v>Operates Crisis lines and resources for victims of domestic violence and general crime.</v>
+      </c>
+      <c r="E172" t="str">
+        <v/>
+      </c>
+      <c r="F172" t="str">
+        <v/>
+      </c>
+      <c r="G172" t="str">
+        <v>9528840376</v>
+      </c>
+      <c r="H172" t="str">
+        <v/>
+      </c>
+      <c r="I172" t="str">
+        <v/>
+      </c>
+      <c r="J172" t="str">
+        <v/>
+      </c>
+      <c r="K172" t="str">
+        <v/>
+      </c>
+      <c r="L172" t="str">
+        <v>https://dayoneservices.org/</v>
+      </c>
+      <c r="M172" t="str">
+        <v>1000 E 80th St. Bloomington, MN 55420</v>
+      </c>
+      <c r="N172" t="str">
+        <v/>
+      </c>
+      <c r="O172" t="str">
+        <v/>
+      </c>
+      <c r="P172" t="str">
+        <v>crime, domestic, violence, sheltering, animals, pet, fostering, hotline, Cornerstone, Day One</v>
+      </c>
+      <c r="Q172" t="str">
+        <v>Cornerstone Website|https://cornerstonemn.org/|link</v>
+      </c>
+      <c r="R172" t="str">
+        <v>Domestic Violence &amp; Safety</v>
+      </c>
+      <c r="S172" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S171"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S172"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -12319,4 +12379,157 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Day One — Sub-Contact Cards</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Each row is a related contact, viewable under the parent Day One resource.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Parent Resource</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sub-Contact Name</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Services / Purpose</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Fax</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Email</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Website</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Location</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Hours / Availability</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Access Instructions</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Day One</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Crisis Hotline</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Hotline</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>1.866.223.1111</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>safety@dayoneservices.org</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>Text line: (612) 399-9995</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Day One</v>
+      </c>
+      <c r="B6" t="str">
+        <v>General Crime Hotline</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>Text Line: (612) 399.9977</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1.866.385.2699</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>safety@dayoneservices.org</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add resource: Planned Parenthood North Central States
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -12,6 +12,7 @@
     <sheet name="SpringPath Mental Heal Contacts" sheetId="7" r:id="rId7"/>
     <sheet name="People Incorporated Contacts" sheetId="8" r:id="rId8"/>
     <sheet name="Day One Contacts" sheetId="9" r:id="rId9"/>
+    <sheet name="Planned Parenthood Nor Contacts" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Screening Tools'!A1:D22</definedName>
@@ -591,9 +592,206 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Planned Parenthood North Central States — Sub-Contact Cards</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Each row is a related contact, viewable under the parent Planned Parenthood North Central States resource.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Parent Resource</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sub-Contact Name</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Services / Purpose</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Fax</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Email</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Website</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Location</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Hours / Availability</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Access Instructions</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Planned Parenthood North Central States</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Brooklyn Park Health Center</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Clinic</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>7635603050</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>https://www.plannedparenthood.org/health-center/minnesota/brooklyn-park/55445/brooklyn-park-clinic-2671-90720</v>
+      </c>
+      <c r="J5" t="str">
+        <v>7532 Brooklyn Blvd., Brooklyn Park, MN 55443</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Monday-Thursday 9AM-6PM, Friday 9AM-5PM, Saturday-Sunday Closed</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Planned Parenthood North Central States</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Eden Prairie Health Center</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Clinic</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>9526534499</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>https://www.plannedparenthood.org/health-center/minnesota/eden-prairie/55344/eden-prairie-clinic-3376-90720</v>
+      </c>
+      <c r="J6" t="str">
+        <v>582 Prairie Center Dr., Suite 215 Eden Prairie, MN 55344</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Monday 8 am - 4 am, Tuesday 10 am - 6 pm, Wednesday 8 am - 4 pm, Thursday 10 am - 6 pm, Friday 8 am - 4 pm, Saturday-Sunday Closed</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Planned Parenthood North Central States</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Minneapolis Health Center</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Clinic</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>6138236300</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>https://www.plannedparenthood.org/health-center/minnesota/minneapolis/55408/minneapolis-clinic-2719-90720</v>
+      </c>
+      <c r="J7" t="str">
+        <v>1200 Lagoon Avenue Minneapolis, MN 55408</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Monday-Friday 9 am - 7 pm, Saturday-Sunday 9 am - 5 pm</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S172"/>
+  <dimension ref="A1:S173"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10755,9 +10953,68 @@
         <v/>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>Planned Parenthood North Central States</v>
+      </c>
+      <c r="B173" t="str">
+        <v>Planned Parenthood</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Family Planning and Health Care Provider</v>
+      </c>
+      <c r="D173" t="str">
+        <v>Provider of Reproductive and Sexual Health care services across the upper-midwest. Services include: Abortion, Birth Control, Emergency Contraception (Morning-After Pill), Gender-Affirming Care, HIV Services, Mental Health, Pregnancy Testing and Planning, Prenatal and Postpartum Services, Sexual and Reproductive Concerns, STD Testing and Treatment, Vaccines, Wellness and Preventive Care</v>
+      </c>
+      <c r="E173" t="str">
+        <v/>
+      </c>
+      <c r="F173" t="str">
+        <v/>
+      </c>
+      <c r="G173" t="str">
+        <v xml:space="preserve"> 1.800.230.7526</v>
+      </c>
+      <c r="H173" t="str">
+        <v/>
+      </c>
+      <c r="I173" t="str">
+        <v/>
+      </c>
+      <c r="J173" t="str">
+        <v/>
+      </c>
+      <c r="K173" t="str">
+        <v/>
+      </c>
+      <c r="L173" t="str">
+        <v>https://www.plannedparenthood.org/planned-parenthood-north-central-states</v>
+      </c>
+      <c r="M173" t="str">
+        <v/>
+      </c>
+      <c r="N173" t="str">
+        <v/>
+      </c>
+      <c r="O173" t="str">
+        <v/>
+      </c>
+      <c r="P173" t="str">
+        <v/>
+      </c>
+      <c r="Q173" t="str">
+        <v/>
+      </c>
+      <c r="R173" t="str">
+        <v>Health Care &amp; Clinics</v>
+      </c>
+      <c r="S173" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S172"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S173"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Edit resource: Planned Parenthood North Central States
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -10953,7 +10953,7 @@
         <v/>
       </c>
     </row>
-    <row r="173">
+    <row r="173" xml:space="preserve">
       <c r="A173" t="str">
         <v>Planned Parenthood North Central States</v>
       </c>
@@ -10963,8 +10963,9 @@
       <c r="C173" t="str">
         <v>Family Planning and Health Care Provider</v>
       </c>
-      <c r="D173" t="str">
-        <v>Provider of Reproductive and Sexual Health care services across the upper-midwest. Services include: Abortion, Birth Control, Emergency Contraception (Morning-After Pill), Gender-Affirming Care, HIV Services, Mental Health, Pregnancy Testing and Planning, Prenatal and Postpartum Services, Sexual and Reproductive Concerns, STD Testing and Treatment, Vaccines, Wellness and Preventive Care</v>
+      <c r="D173" t="str" xml:space="preserve">
+        <v xml:space="preserve">Provider of Reproductive and Sexual Health care services across the upper-midwest. Services include: Abortion, Birth Control, Emergency Contraception (Morning-After Pill), Gender-Affirming Care, HIV Services, Mental Health, Pregnancy Testing and Planning, Prenatal and Postpartum Services, Sexual and Reproductive Concerns, STD Testing and Treatment, Vaccines, Wellness and Preventive Care
+In-person and telehealth appointments are available.</v>
       </c>
       <c r="E173" t="str">
         <v/>
@@ -11000,7 +11001,7 @@
         <v/>
       </c>
       <c r="P173" t="str">
-        <v/>
+        <v>Planned Parenthood, sexual, reproductive, mental health, abortion, HIV, AIDS, STD, testing, telehealth</v>
       </c>
       <c r="Q173" t="str">
         <v/>

</xml_diff>

<commit_message>
Add resource: Jewish Family and Children's Service of Minnesota
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -13,6 +13,7 @@
     <sheet name="People Incorporated Contacts" sheetId="8" r:id="rId8"/>
     <sheet name="Day One Contacts" sheetId="9" r:id="rId9"/>
     <sheet name="Planned Parenthood Nor Contacts" sheetId="10" r:id="rId10"/>
+    <sheet name="Jewish Family and Chil Contacts" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Screening Tools'!A1:D22</definedName>
@@ -789,9 +790,118 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Jewish Family and Children's Service of Minnesota — Sub-Contact Cards</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Each row is a related contact, viewable under the parent Jewish Family and Children's Service of Minnesota resource.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Parent Resource</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sub-Contact Name</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Services / Purpose</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Fax</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Email</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Website</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Location</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Hours / Availability</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Access Instructions</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Jewish Family and Children's Service of Minnesota</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Intake &amp; Resource Connection</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>JFCS’ first response to questions or requests for help.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>952-542-4843</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>intake@jfcsmn.org</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://www.jfcsmn.org/help/</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S173"/>
+  <dimension ref="A1:S174"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11013,9 +11123,68 @@
         <v/>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>Jewish Family and Children's Service of Minnesota</v>
+      </c>
+      <c r="B174" t="str">
+        <v>JFCS</v>
+      </c>
+      <c r="C174" t="str">
+        <v xml:space="preserve">Religious Non-Profit </v>
+      </c>
+      <c r="D174" t="str">
+        <v>Services include counseling and mental heath services, transportation, case management, senior companionship, and kosher meals on wheels, and more.</v>
+      </c>
+      <c r="E174" t="str">
+        <v/>
+      </c>
+      <c r="F174" t="str">
+        <v>jfcs@jfcsmn.org</v>
+      </c>
+      <c r="G174" t="str">
+        <v>9525460616</v>
+      </c>
+      <c r="H174" t="str">
+        <v/>
+      </c>
+      <c r="I174" t="str">
+        <v>9525931778</v>
+      </c>
+      <c r="J174" t="str">
+        <v/>
+      </c>
+      <c r="K174" t="str">
+        <v/>
+      </c>
+      <c r="L174" t="str">
+        <v>https://www.jfcsmn.org/</v>
+      </c>
+      <c r="M174" t="str">
+        <v>5905 Golden Valley Rd, Golden Valley, MN 55422</v>
+      </c>
+      <c r="N174" t="str">
+        <v/>
+      </c>
+      <c r="O174" t="str">
+        <v>Monday-Tuesday 8:30 am to 5:00 pm, Wednesday 8:30 am to 7:00 pm, Thursday  8:30 am to 5:00 pm, Friday 8:30 am to 4:00 pm</v>
+      </c>
+      <c r="P174" t="str">
+        <v/>
+      </c>
+      <c r="Q174" t="str">
+        <v>Garber Transportation Flyer|Garber_Transportation_Overview_26.pdf; Accompanied Transportation Services flyer|Accompanied-Transportation-Services_flyer.pdf; Care Planning Consultation flyer|Care-Planning-Consultation_flyer.pdf; Case Management flyer|Case-Management_flyer.pdf; Dementia Caregiver Connect flyer|Dementia-Caregiver-Connect-flyer.pdf; Dementia Friends Flyer|Dementia-Friends-Flyer_24.pdf; Holocaust Survivor flyer|Holocaust-Survivor_flyer.pdf; Kosher Meals On Wheels flyer|MOW-flyer_26.pdf; MemoryCafe flyer|MemoryCafe-flyer_25.pdf; Shopping Services flyer|Shopping-Services_flyer.pdf; Recovery Resource Guide|Recovery-Resource-Guide.pdf; Garber Transportation Inquiry Form|https://www.jfcsmn.org/garber-transportation-program-inquiry/|link</v>
+      </c>
+      <c r="R174" t="str">
+        <v>Immigrant / Culturally Specific</v>
+      </c>
+      <c r="S174" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S173"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S174"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Edit resource: Domestic Abuse Service Center
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -2043,13 +2043,13 @@
       <c r="F20" t="str">
         <v/>
       </c>
-      <c r="G20">
+      <c r="G20" t="str">
         <v>6123485073</v>
       </c>
       <c r="H20" t="str">
         <v/>
       </c>
-      <c r="I20">
+      <c r="I20" t="str">
         <v>6123485892</v>
       </c>
       <c r="J20" t="str">
@@ -2068,7 +2068,7 @@
         <v/>
       </c>
       <c r="O20" t="str">
-        <v/>
+        <v xml:space="preserve">Monday – Friday 8:00 am to 4:30 pm  </v>
       </c>
       <c r="P20" t="str">
         <v>domestic, abuse, service, center, protection, orders, legal, advocacy, safety, planning, housing, referrals</v>
@@ -2080,7 +2080,7 @@
         <v>Domestic Violence &amp; Safety</v>
       </c>
       <c r="S20" t="str">
-        <v>domestic; abuse; service; center; protection; orders; legal; advocacy; safety; planning; housing; referrals</v>
+        <v/>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Add resource: Vail Communities
</commit_message>
<xml_diff>
--- a/ARM-Builder/New_ARM_Library.xlsx
+++ b/ARM-Builder/New_ARM_Library.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Day One Contacts" sheetId="9" r:id="rId9"/>
     <sheet name="Planned Parenthood Nor Contacts" sheetId="10" r:id="rId10"/>
     <sheet name="Jewish Family and Chil Contacts" sheetId="11" r:id="rId11"/>
+    <sheet name="Vail Communities Contacts" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Screening Tools'!A1:D22</definedName>
@@ -899,9 +900,210 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Vail Communities — Sub-Contact Cards</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Each row is a related contact, viewable under the parent Vail Communities resource.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Parent Resource</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sub-Contact Name</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Services / Purpose</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Fax</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Email</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Website</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Location</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Hours / Availability</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Access Instructions</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Vail Communities</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Targeted Case Management</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Case Management</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>(952) 945-4275</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>kfaber@vailcommunities.org</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://vailcommunities.org/targeted-case-management</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>Contact information is for Kristen Farber, Case Management Program Assistant.</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>Vail Communities</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Hopkins Clubhouse</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Day Program</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>(952) 297-8908</v>
+      </c>
+      <c r="G6" t="str">
+        <v>952) 938-7934</v>
+      </c>
+      <c r="H6" t="str">
+        <v>nroehl@vailcommunities.org</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://vailcommunities.org/hopkins-clubhouse</v>
+      </c>
+      <c r="J6" t="str">
+        <v>15 9th Ave S., Hopkins, MN 55343</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Mon-Fri 8:30a-4:30p, Open until 6:30p on Thursday Evenings</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Intake Coordinator
+Nikki Roehl (she/her)
+Phone: 952-300-5378</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>Vail Communities</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Uptown Clubhouse</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Day Program</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>952) 297-8900</v>
+      </c>
+      <c r="G7" t="str">
+        <v>(952) 938-7934</v>
+      </c>
+      <c r="H7" t="str">
+        <v>eisaacson@vailcommunities.org</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://vailcommunities.org/uptown-clubhouse</v>
+      </c>
+      <c r="J7" t="str">
+        <v>1412 W. 36th St., Mpls, MN 55408</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Mon-Fri 8:30a-4:30p, Open until 6:30p on Wednesday Evenings</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Intake Coordinator
+Elaine Isaacson (she/her)
+Phone: 612-760-3147</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S174"/>
+  <dimension ref="A1:S175"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11182,9 +11384,69 @@
         <v/>
       </c>
     </row>
+    <row r="175" xml:space="preserve">
+      <c r="A175" t="str">
+        <v>Vail Communities</v>
+      </c>
+      <c r="B175" t="str">
+        <v>Vail Communities</v>
+      </c>
+      <c r="C175" t="str">
+        <v>Nonprofit Mental Health Services</v>
+      </c>
+      <c r="D175" t="str" xml:space="preserve">
+        <v xml:space="preserve">Nonprofit organization that provides community-based recovery services for adults with serious mental illnesses. Programs include clubhouses, targeted case management, and Assertive Outreach.
+ </v>
+      </c>
+      <c r="E175" t="str">
+        <v/>
+      </c>
+      <c r="F175" t="str">
+        <v>info@vailcommunities.org</v>
+      </c>
+      <c r="G175" t="str">
+        <v>952-938-9622</v>
+      </c>
+      <c r="H175" t="str">
+        <v/>
+      </c>
+      <c r="I175" t="str">
+        <v/>
+      </c>
+      <c r="J175" t="str">
+        <v/>
+      </c>
+      <c r="K175" t="str">
+        <v/>
+      </c>
+      <c r="L175" t="str">
+        <v>https://vailcommunities.org/</v>
+      </c>
+      <c r="M175" t="str">
+        <v>23 9th Ave. S., Hopkins, MN 55343</v>
+      </c>
+      <c r="N175" t="str">
+        <v/>
+      </c>
+      <c r="O175" t="str">
+        <v/>
+      </c>
+      <c r="P175" t="str">
+        <v>Vail, Communities, Day program, clubhouse, mental health, Targeted, case management, AOC</v>
+      </c>
+      <c r="Q175" t="str">
+        <v>AOS Brochure|AOS_Brochure_Tri_Fold_Final.pdf</v>
+      </c>
+      <c r="R175" t="str">
+        <v>Mental Health &amp; Substance Use</v>
+      </c>
+      <c r="S175" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S174"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S175"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>